<commit_message>
Fix pipeline cost bug
</commit_message>
<xml_diff>
--- a/adopt_net0/database/data/networks/co2_transport_oeuvray/OtherData.xlsx
+++ b/adopt_net0/database/data/networks/co2_transport_oeuvray/OtherData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\6574114\PycharmProjects\AdOpT_TechnologyDatabase\technology_database\networks\data\co2_pipeline\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwiegner\PycharmProjects\AdOpT_DAC-Offshore\adopt_net0\database\data\networks\co2_transport_oeuvray\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADBA3B20-1076-4FE7-92FC-401996B35FCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7890D27A-E9B9-456E-819B-C8592E432328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Universal" sheetId="1" r:id="rId1"/>
@@ -532,13 +532,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -554,7 +554,7 @@
         <v>5.0000000000000002E-5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -562,7 +562,7 @@
         <v>9.81</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -570,7 +570,7 @@
         <v>8.31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -578,7 +578,7 @@
         <v>4.4010000000000001E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -586,7 +586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -594,7 +594,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -602,7 +602,7 @@
         <v>7900</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -610,25 +610,23 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>25</v>
       </c>
       <c r="B10">
-        <f>1.5/100</f>
-        <v>1.4999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>26</v>
       </c>
       <c r="B11">
-        <f>4/100</f>
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+        <v>1.4999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -636,7 +634,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>48</v>
       </c>
@@ -644,7 +642,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>49</v>
       </c>
@@ -652,7 +650,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -660,7 +658,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -668,7 +666,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -676,7 +674,7 @@
         <v>110000</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -684,7 +682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -692,7 +690,7 @@
         <v>1000000000000</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -701,7 +699,7 @@
         <v>1.8304642670839855</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -709,7 +707,7 @@
         <v>1013.1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -717,7 +715,7 @@
         <v>7900</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>46</v>
       </c>
@@ -725,7 +723,7 @@
         <v>2.04</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>47</v>
       </c>
@@ -741,9 +739,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B34D0E1F-EF3B-480B-BA74-58FDE3E1D36B}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -751,7 +749,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>50</v>
       </c>
@@ -759,7 +757,7 @@
         <v>21900000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>51</v>
       </c>
@@ -767,7 +765,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -775,7 +773,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>54</v>
       </c>
@@ -783,7 +781,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>53</v>
       </c>
@@ -799,9 +797,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E688A991-2A6E-446B-8C7D-F1CA6357E4CA}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -809,7 +807,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>55</v>
       </c>
@@ -817,7 +815,7 @@
         <v>74300</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>56</v>
       </c>
@@ -833,9 +831,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45044F5A-A9E9-4945-9CB2-571E515056E3}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -846,7 +844,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -857,7 +855,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -868,7 +866,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -879,7 +877,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -890,7 +888,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>45</v>
       </c>
@@ -901,7 +899,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -912,7 +910,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -923,7 +921,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -934,18 +932,18 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
       <c r="B10">
-        <v>0.72</v>
+        <v>0.5</v>
       </c>
       <c r="C10">
         <v>0.61</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>42</v>
       </c>
@@ -964,9 +962,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A45B4FD2-4527-4060-960E-3ED97ED5C802}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -977,7 +978,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -988,7 +989,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -999,7 +1000,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -1010,7 +1011,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -1021,7 +1022,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>45</v>
       </c>
@@ -1032,7 +1033,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1043,7 +1044,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -1054,7 +1055,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -1065,18 +1066,18 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
       <c r="B10">
-        <v>0.72</v>
+        <v>0.5</v>
       </c>
       <c r="C10">
         <v>0.61</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>42</v>
       </c>
@@ -1095,9 +1096,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16922DF8-7098-4044-8DE1-B80EBC856B23}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -1117,7 +1118,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1137,7 +1138,7 @@
         <v>1.17</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1157,7 +1158,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1177,7 +1178,7 @@
         <v>1.37</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1197,7 +1198,7 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1217,7 +1218,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1237,7 +1238,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -1257,7 +1258,7 @@
         <v>1.54</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1285,9 +1286,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEC8EA4E-6A3C-4C09-A1E7-AD509FB86A4E}">
   <dimension ref="A1:X2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -1361,7 +1362,7 @@
         <v>1.42</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>

</xml_diff>